<commit_message>
fix(craft): prioritize quest candidate recipes and sync spirit summon materials
</commit_message>
<xml_diff>
--- a/balance/Spiria_Game_spirit.xlsx
+++ b/balance/Spiria_Game_spirit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dawoonkim/Desktop/spiria game/balance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92D94C6-03BF-DA49-B274-4815C35B1B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BCB2F32-2126-0E42-95B3-F65192996B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="27860" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="34200" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="정령·의뢰서 합본" sheetId="1" r:id="rId1"/>
@@ -210,9 +210,6 @@
     <t>“오늘은 네 마음에 어떤 꽃을 피워 볼까?”</t>
   </si>
   <si>
-    <t xml:space="preserve">물 → 달 → 별 </t>
-  </si>
-  <si>
     <t>플레오</t>
   </si>
   <si>
@@ -956,6 +953,10 @@
 꽃잎에 깃든 신비로운 기운이 
 빛을 붙잡고 있는 걸까요, 
 아니면 달빛 비친 호수에 별빛이 스며든 걸까요?</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">달 → 별 → 에테르 </t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1744,7 +1745,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C2" s="17" t="s">
         <v>22</v>
@@ -1765,7 +1766,7 @@
         <v>27</v>
       </c>
       <c r="I2" s="16" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J2" s="16" t="s">
         <v>28</v>
@@ -1780,7 +1781,7 @@
         <v>94</v>
       </c>
       <c r="N2" s="17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O2" s="21">
         <v>74</v>
@@ -1798,13 +1799,13 @@
         <v>34</v>
       </c>
       <c r="T2" s="45" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="U2" s="45" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="V2" s="45" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="91.5" customHeight="1">
@@ -1812,7 +1813,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C3" s="25" t="s">
         <v>35</v>
@@ -1833,7 +1834,7 @@
         <v>38</v>
       </c>
       <c r="I3" s="26" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J3" s="26" t="s">
         <v>39</v>
@@ -1866,13 +1867,13 @@
         <v>45</v>
       </c>
       <c r="T3" s="45" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="U3" s="45" t="s">
+        <v>205</v>
+      </c>
+      <c r="V3" s="45" t="s">
         <v>206</v>
-      </c>
-      <c r="V3" s="45" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="91.5" customHeight="1">
@@ -1880,7 +1881,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C4" s="34" t="s">
         <v>46</v>
@@ -1901,7 +1902,7 @@
         <v>49</v>
       </c>
       <c r="I4" s="33" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="J4" s="33" t="s">
         <v>50</v>
@@ -1934,13 +1935,13 @@
         <v>56</v>
       </c>
       <c r="T4" s="45" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="U4" s="45" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="V4" s="45" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="91.5" customHeight="1">
@@ -1948,67 +1949,67 @@
         <v>4</v>
       </c>
       <c r="B5" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="C5" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="D5" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="E5" s="26" t="s">
         <v>59</v>
-      </c>
-      <c r="E5" s="26" t="s">
-        <v>60</v>
       </c>
       <c r="F5" s="24" t="s">
         <v>25</v>
       </c>
       <c r="G5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="H5" s="26" t="s">
+      <c r="I5" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="J5" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="26" t="s">
-        <v>224</v>
-      </c>
-      <c r="J5" s="26" t="s">
+      <c r="K5" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="K5" s="26" t="s">
-        <v>64</v>
-      </c>
       <c r="L5" s="27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M5" s="28">
         <v>94</v>
       </c>
       <c r="N5" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O5" s="30">
         <v>73</v>
       </c>
       <c r="P5" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q5" s="43" t="s">
         <v>66</v>
       </c>
-      <c r="Q5" s="43" t="s">
+      <c r="R5" s="44" t="s">
+        <v>185</v>
+      </c>
+      <c r="S5" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="R5" s="44" t="s">
+      <c r="T5" s="45" t="s">
         <v>186</v>
       </c>
-      <c r="S5" s="43" t="s">
-        <v>68</v>
-      </c>
-      <c r="T5" s="45" t="s">
-        <v>187</v>
-      </c>
       <c r="U5" s="45" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="V5" s="45" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:22" ht="91.5" customHeight="1">
@@ -2016,7 +2017,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" s="29" t="s">
         <v>41</v>
@@ -2025,22 +2026,22 @@
         <v>23</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F6" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H6" s="16" t="s">
         <v>27</v>
       </c>
       <c r="I6" s="26" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K6" s="16" t="s">
         <v>29</v>
@@ -2058,25 +2059,25 @@
         <v>74</v>
       </c>
       <c r="P6" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q6" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="Q6" s="44" t="s">
+      <c r="R6" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="R6" s="43" t="s">
+      <c r="S6" s="43" t="s">
         <v>74</v>
       </c>
-      <c r="S6" s="43" t="s">
-        <v>75</v>
-      </c>
       <c r="T6" s="45" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="U6" s="45" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="V6" s="45" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="91.5" customHeight="1">
@@ -2084,37 +2085,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="D7" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="E7" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="E7" s="33" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" s="36" t="s">
+      <c r="G7" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="H7" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="H7" s="33" t="s">
+      <c r="I7" s="33" t="s">
+        <v>226</v>
+      </c>
+      <c r="J7" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="I7" s="33" t="s">
-        <v>227</v>
-      </c>
-      <c r="J7" s="33" t="s">
+      <c r="K7" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="K7" s="33" t="s">
-        <v>83</v>
-      </c>
       <c r="L7" s="37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M7" s="38">
         <v>96</v>
@@ -2126,25 +2127,25 @@
         <v>75</v>
       </c>
       <c r="P7" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q7" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="Q7" s="44" t="s">
+      <c r="R7" s="43" t="s">
         <v>85</v>
       </c>
-      <c r="R7" s="43" t="s">
+      <c r="S7" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="S7" s="44" t="s">
-        <v>87</v>
-      </c>
       <c r="T7" s="45" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="U7" s="45" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="V7" s="45" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="91.5" customHeight="1">
@@ -2152,37 +2153,37 @@
         <v>7</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C8" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="26" t="s">
         <v>88</v>
-      </c>
-      <c r="D8" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="26" t="s">
-        <v>89</v>
       </c>
       <c r="F8" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G8" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="H8" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="H8" s="26" t="s">
+      <c r="I8" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="J8" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="I8" s="26" t="s">
-        <v>228</v>
-      </c>
-      <c r="J8" s="26" t="s">
+      <c r="K8" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="K8" s="26" t="s">
-        <v>93</v>
-      </c>
       <c r="L8" s="27" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M8" s="28">
         <v>95</v>
@@ -2194,25 +2195,25 @@
         <v>74</v>
       </c>
       <c r="P8" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q8" s="43" t="s">
         <v>94</v>
       </c>
-      <c r="Q8" s="43" t="s">
+      <c r="R8" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="R8" s="44" t="s">
-        <v>96</v>
-      </c>
       <c r="S8" s="44" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="T8" s="45" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U8" s="45" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="V8" s="45" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="91.5" customHeight="1">
@@ -2220,34 +2221,34 @@
         <v>8</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>30</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F9" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G9" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="H9" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="H9" s="26" t="s">
+      <c r="I9" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="J9" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I9" s="26" t="s">
-        <v>229</v>
-      </c>
-      <c r="J9" s="26" t="s">
+      <c r="K9" s="26" t="s">
         <v>100</v>
-      </c>
-      <c r="K9" s="26" t="s">
-        <v>101</v>
       </c>
       <c r="L9" s="27" t="s">
         <v>30</v>
@@ -2262,25 +2263,25 @@
         <v>73</v>
       </c>
       <c r="P9" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q9" s="43" t="s">
         <v>102</v>
       </c>
-      <c r="Q9" s="43" t="s">
+      <c r="R9" s="43" t="s">
         <v>103</v>
       </c>
-      <c r="R9" s="43" t="s">
+      <c r="S9" s="44" t="s">
         <v>104</v>
       </c>
-      <c r="S9" s="44" t="s">
-        <v>105</v>
-      </c>
       <c r="T9" s="45" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="U9" s="45" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="V9" s="45" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="91.5" customHeight="1">
@@ -2288,7 +2289,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C10" s="34" t="s">
         <v>52</v>
@@ -2297,25 +2298,25 @@
         <v>23</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G10" s="42" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" s="33" t="s">
         <v>106</v>
       </c>
-      <c r="H10" s="33" t="s">
+      <c r="I10" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="J10" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="I10" s="33" t="s">
-        <v>232</v>
-      </c>
-      <c r="J10" s="33" t="s">
+      <c r="K10" s="33" t="s">
         <v>108</v>
-      </c>
-      <c r="K10" s="33" t="s">
-        <v>109</v>
       </c>
       <c r="L10" s="37" t="s">
         <v>52</v>
@@ -2324,31 +2325,31 @@
         <v>94</v>
       </c>
       <c r="N10" s="34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O10" s="39">
         <v>76</v>
       </c>
       <c r="P10" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q10" s="44" t="s">
         <v>110</v>
       </c>
-      <c r="Q10" s="44" t="s">
+      <c r="R10" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="R10" s="44" t="s">
+      <c r="S10" s="44" t="s">
         <v>112</v>
       </c>
-      <c r="S10" s="44" t="s">
-        <v>113</v>
-      </c>
       <c r="T10" s="45" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="U10" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="V10" s="45" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="91.5" customHeight="1">
@@ -2356,67 +2357,67 @@
         <v>10</v>
       </c>
       <c r="B11" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="D11" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="26" t="s">
         <v>115</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>116</v>
       </c>
       <c r="F11" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G11" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="H11" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="H11" s="26" t="s">
+      <c r="I11" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="J11" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="I11" s="26" t="s">
-        <v>237</v>
-      </c>
-      <c r="J11" s="26" t="s">
+      <c r="K11" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="K11" s="26" t="s">
-        <v>120</v>
-      </c>
       <c r="L11" s="27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M11" s="28">
         <v>94</v>
       </c>
       <c r="N11" s="29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O11" s="30">
         <v>71</v>
       </c>
       <c r="P11" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q11" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="Q11" s="43" t="s">
+      <c r="R11" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="R11" s="44" t="s">
+      <c r="S11" s="43" t="s">
         <v>124</v>
       </c>
-      <c r="S11" s="43" t="s">
-        <v>125</v>
-      </c>
       <c r="T11" s="45" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="U11" s="45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="V11" s="45" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="91.5" customHeight="1">
@@ -2424,67 +2425,67 @@
         <v>11</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E12" s="26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G12" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="H12" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="H12" s="26" t="s">
+      <c r="I12" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="J12" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="I12" s="26" t="s">
-        <v>235</v>
-      </c>
-      <c r="J12" s="26" t="s">
+      <c r="K12" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="K12" s="26" t="s">
-        <v>129</v>
-      </c>
       <c r="L12" s="27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M12" s="28">
         <v>95</v>
       </c>
       <c r="N12" s="29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O12" s="30">
         <v>72</v>
       </c>
       <c r="P12" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q12" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="Q12" s="43" t="s">
+      <c r="R12" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="R12" s="43" t="s">
+      <c r="S12" s="43" t="s">
         <v>132</v>
       </c>
-      <c r="S12" s="43" t="s">
-        <v>133</v>
-      </c>
       <c r="T12" s="45" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="U12" s="45" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="V12" s="45" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="91.5" customHeight="1">
@@ -2492,67 +2493,67 @@
         <v>12</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D13" s="33" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F13" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="G13" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="G13" s="33" t="s">
+      <c r="H13" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="H13" s="33" t="s">
+      <c r="I13" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="J13" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="I13" s="33" t="s">
-        <v>236</v>
-      </c>
-      <c r="J13" s="33" t="s">
+      <c r="K13" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="K13" s="33" t="s">
-        <v>138</v>
-      </c>
       <c r="L13" s="37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M13" s="38">
         <v>98</v>
       </c>
       <c r="N13" s="34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O13" s="39">
         <v>69</v>
       </c>
       <c r="P13" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q13" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="Q13" s="43" t="s">
+      <c r="R13" s="43" t="s">
         <v>140</v>
       </c>
-      <c r="R13" s="43" t="s">
+      <c r="S13" s="43" t="s">
         <v>141</v>
       </c>
-      <c r="S13" s="43" t="s">
-        <v>142</v>
-      </c>
       <c r="T13" s="45" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="U13" s="45" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="V13" s="45" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2593,7 +2594,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1">
       <c r="A1" s="46" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
@@ -2601,170 +2602,170 @@
     </row>
     <row r="3" spans="1:4" ht="18" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="36" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>148</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>149</v>
       </c>
       <c r="C4" s="5">
         <v>30</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="5">
         <v>15</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C6" s="5">
         <v>15</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C7" s="5">
         <v>10</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>157</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>158</v>
       </c>
       <c r="C8" s="5">
         <v>15</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C9" s="5">
         <v>10</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1">
       <c r="A10" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>167</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>170</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>173</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1">
       <c r="A14" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="17" customHeight="1">
@@ -2775,52 +2776,52 @@
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1">
       <c r="A16" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>178</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>179</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1">
       <c r="A17" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>182</v>
-      </c>
       <c r="C17" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="18" customHeight="1">
       <c r="A18" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>184</v>
-      </c>
       <c r="C18" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="36" customHeight="1">
       <c r="A19" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="13"/>

</xml_diff>